<commit_message>
Refined quarterly invoice SKILL
</commit_message>
<xml_diff>
--- a/.claude/skills/invoice-tracker/output/cost_tracker.xlsx
+++ b/.claude/skills/invoice-tracker/output/cost_tracker.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Line Items'!$A$1:$O$105</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anomalies'!$A$1:$G$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anomalies'!$A$1:$G$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8952,7 +8952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9184,30 +9184,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>13.85</v>
+        <v>16.38</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Charged 23/04/2025 (36 days before period start); period 29/05/2025-28/08/2025. "Attended site to re-fit fan control cabinet to the wall: 26/"</t>
+          <t>Maintenance: 20.40 this quarter vs prior average 4.02 (5.1x, higher).</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9220,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>1883739</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -9234,15 +9230,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-1.03</v>
+        <v>13.85</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Charged 01/07/2025 (59 days before period start); period 29/08/2025-28/11/2025. "Attended site to program numbers as requested"</t>
+          <t>Charged 23/04/2025 (36 days before period start); period 29/05/2025-28/08/2025. "Attended site to re-fit fan control cabinet to the wall: 26/"</t>
         </is>
       </c>
     </row>
@@ -9269,15 +9265,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>3.4</v>
+        <v>-1.03</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Charged 15/07/2025 (45 days before period start); period 29/08/2025-28/11/2025. "Monitoring of CCTV"</t>
+          <t>Charged 01/07/2025 (59 days before period start); period 29/08/2025-28/11/2025. "Attended site to program numbers as requested"</t>
         </is>
       </c>
     </row>
@@ -9304,15 +9300,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ONESCO Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>11.03</v>
+        <v>3.4</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Charged 17/07/2025 (43 days before period start); period 29/08/2025-28/11/2025. "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2025"</t>
+          <t>Charged 15/07/2025 (45 days before period start); period 29/08/2025-28/11/2025. "Monitoring of CCTV"</t>
         </is>
       </c>
     </row>
@@ -9329,25 +9325,25 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>ONESCO Ltd</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>86.5</v>
+        <v>11.03</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Charged 28/05/2026 (89 days after period end); period 29/11/2025-28/02/2026. "Management Fee: 01/03/2026 - 28/05/2026"</t>
+          <t>Charged 17/07/2025 (43 days before period start); period 29/08/2025-28/11/2025. "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2025"</t>
         </is>
       </c>
     </row>
@@ -9364,25 +9360,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Life System</t>
+          <t>Management Fee</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>2.7</v>
+        <v>86.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Charged 17/12/2025 (74 days before period start); period 01/03/2026-28/05/2026. "Quarterly fire alarm service"</t>
+          <t>Charged 28/05/2026 (89 days after period end); period 29/11/2025-28/02/2026. "Management Fee: 01/03/2026 - 28/05/2026"</t>
         </is>
       </c>
     </row>
@@ -9404,7 +9400,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -9413,11 +9409,11 @@
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1.03</v>
+        <v>2.7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Charged 23/12/2025 (68 days before period start); period 01/03/2026-28/05/2026. "Door entry sim card change"</t>
+          <t>Charged 17/12/2025 (74 days before period start); period 01/03/2026-28/05/2026. "Quarterly fire alarm service"</t>
         </is>
       </c>
     </row>
@@ -9444,15 +9440,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ritchie Mackenzie &amp; Co Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>58.58</v>
+        <v>1.03</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Charged 28/01/2026 (32 days before period start); period 01/03/2026-28/05/2026. "Attended site to install new pump to replace missing pump"</t>
+          <t>Charged 23/12/2025 (68 days before period start); period 01/03/2026-28/05/2026. "Door entry sim card change"</t>
         </is>
       </c>
     </row>
@@ -9474,20 +9470,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>Ritchie Mackenzie &amp; Co Ltd</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>86.5</v>
+        <v>58.58</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Charged 28/08/2026 (92 days after period end); period 01/03/2026-28/05/2026. "Management Fee: 29/05/2026 - 28/08/2026"</t>
+          <t>Charged 28/01/2026 (32 days before period start); period 01/03/2026-28/05/2026. "Attended site to install new pump to replace missing pump"</t>
         </is>
       </c>
     </row>
@@ -9499,7 +9495,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -9507,15 +9503,22 @@
           <t>2013624</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ASD Electrical Contractors Ltd</t>
-        </is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>86.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>'ASD Electrical Contractors Ltd' billed in 3/3 prior quarters but is absent this quarter.</t>
+          <t>Charged 28/08/2026 (92 days after period end); period 01/03/2026-28/05/2026. "Management Fee: 29/05/2026 - 28/08/2026"</t>
         </is>
       </c>
     </row>
@@ -9527,26 +9530,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New vendor</t>
+          <t>Dropped vendor</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Argyle Locksmiths</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>2.71</v>
+          <t>HDN- NIG - 2025-2026</t>
+        </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>'Argyle Locksmiths' appears this quarter but not in any prior quarter (cost 2.71).</t>
+          <t>'HDN- NIG - 2025-2026' billed in 2/2 prior quarters but is absent this quarter.</t>
         </is>
       </c>
     </row>
@@ -9558,30 +9558,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Stale service period</t>
+          <t>Dropped vendor</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1883739</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>13.85</v>
+          <t>ASD Electrical Contractors Ltd</t>
+        </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Service period 26/03/2025-23/04/2025 ends 36 days before the invoice quarter starts (29/05/2025). "Attended site to re-fit fan control cabinet to the"</t>
+          <t>'ASD Electrical Contractors Ltd' billed in 3/3 prior quarters but is absent this quarter.</t>
         </is>
       </c>
     </row>
@@ -9593,7 +9586,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Stale service period</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9601,959 +9594,824 @@
           <t>1933254</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ONESCO Ltd</t>
+          <t>AB Decorators</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.03</v>
+        <v>22.29</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Service period 26/06/2025-17/07/2025 ends 43 days before the invoice quarter starts (29/08/2025). "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2"</t>
+          <t>'AB Decorators' appears this quarter but not in any prior quarter (cost 22.29).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abnormal category total</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Electricity</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Columbus Facilities Maintenance Ltd</t>
+        </is>
+      </c>
       <c r="F20" s="3" t="n">
-        <v>-120.6166666666667</v>
+        <v>18.85</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Electricity: 84.61 this quarter vs prior average 205.23 (0.4x, lower).</t>
+          <t>'Columbus Facilities Maintenance Ltd' appears this quarter but not in any prior quarter (cost 18.85).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Abnormal vendor total</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
+          <t>Hart Lifts Ltd</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>'Hart Lifts Ltd' appears this quarter but not in any prior quarter (cost 7.52).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Integra Building Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>'Integra Building Solutions Ltd' appears this quarter but not in any prior quarter (cost 2.23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ONESCO Ltd</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>44.27</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>'ONESCO Ltd' appears this quarter but not in any prior quarter (cost 44.27).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PTSG Electrical Services Ltd</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>'PTSG Electrical Services Ltd' appears this quarter but not in any prior quarter (cost 22.94).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>APS Safety Systems Limited</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>'APS Safety Systems Limited' appears this quarter but not in any prior quarter (cost 10.51).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>City Drain Clear</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>'City Drain Clear' appears this quarter but not in any prior quarter (cost 3.34).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Cleansite Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>'Cleansite Solutions Ltd' appears this quarter but not in any prior quarter (cost 5.15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>DAWN ZURICH 26/27</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>'DAWN ZURICH 26/27' appears this quarter but not in any prior quarter (cost 11.43).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>DAWN- INTACT-26-27</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>181.01</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>'DAWN- INTACT-26-27' appears this quarter but not in any prior quarter (cost 181.01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>J.T. Mullen Building Services</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>'J.T. Mullen Building Services' appears this quarter but not in any prior quarter (cost 3.77).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>New vendor</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Argyle Locksmiths</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>'Argyle Locksmiths' appears this quarter but not in any prior quarter (cost 2.71).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>'attended site and downloaded cctv footage from mailbox camera' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>'attended site and removed snib from fire door dry riser door was detached from wall so attached timber batons to secure door' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>'attended site to re fit fan control cabinet to the wall' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>'emergency lighting repair' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>'quarterly service and inspection car park garage shutter' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>'replace faulty ball valves' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>'service checks of x booster set' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>'sim card charge for the gsm door access system' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>'sim card charges for gsm door access system' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>'vecon drive at pump' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>'water testing certification' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>'attended site to program numbers as requested' (e.g. Repairs) appeared in all 2 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>'quarterly fire alarm service' (e.g. Life System) appeared in all 2 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Stale service period</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
-        <v>42.92666666666666</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd: 81.91 this quarter vs prior average 38.98 (2.1x, higher).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1883739</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Charged 30/04/2025 (29 days before period start); period 29/05/2025-28/08/2025. "Sim card charge for the GSM door access system: 01/04/2025 -"</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1883739</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Charged 23/05/2025 (6 days before period start); period 29/05/2025-28/08/2025. "Attended site and downloaded CCTV footage from mailbox camer"</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1883739</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>80.28</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Charged 29/08/2025 (1 days after period end); period 29/05/2025-28/08/2025. "Management Fee: 29/08/2025 - 28/11/2025"</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="F45" s="3" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Service period 26/03/2025-23/04/2025 ends 36 days before the invoice quarter starts (29/05/2025). "Attended site to re-fit fan control cabinet to the"</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Stale service period</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
         <is>
           <t>1933254</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>PTSG Electrical Services Ltd</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Charged 08/08/2025 (21 days before period start); period 29/08/2025-28/11/2025. "Test &amp; Inspection of the Lighting Protection System"</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Charged 22/08/2025 (7 days before period start); period 29/08/2025-28/11/2025. "Door entry SIM card charge"</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Repairs</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>AB Decorators</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>22.29</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Charged 26/08/2025 (3 days before period start); period 29/08/2025-28/11/2025. "Repairs to floor 11, 4, 1 &amp; stairwell to ground"</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>-7.42</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025. "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>80.28</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025. "Management Fee: 29/11/2025 - 28/02/2026"</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Grounds</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Cleansite Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Charged 17/11/2025 (12 days before period start); period 29/11/2025-28/02/2026. "Bulk uplift"</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Ritchie Mackenzie &amp; Co Ltd</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>5.83</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Charged 31/10/2025 (29 days before period start); period 29/11/2025-28/02/2026. "Service checks on 1 x Two Pump Booster Set"</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Hart Lifts Ltd</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Charged 14/11/2025 (15 days before period start); period 29/11/2025-28/02/2026. "Repairs to lift controller unit"</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Hart Lifts Ltd</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Charged 21/11/2025 (8 days before period start); period 29/11/2025-28/02/2026. "Renewed damaged lift door spring"</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Integra Building Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="n">
-        <v>2.57</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Charged 25/11/2025 (4 days before period start); period 29/11/2025-28/02/2026. "Replace dry riser inlet lock"</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="n">
-        <v>-7.72</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Charged 01/03/2026 (1 days after period end); period 29/11/2025-28/02/2026. "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Charged 31/01/2026 (29 days before period start); period 01/03/2026-28/05/2026. "Door entry SIM card charge"</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Charged 15/02/2026 (14 days before period start); period 01/03/2026-28/05/2026. "Reset fire alarm system"</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Hart Lifts Ltd</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Charged 30/01/2026 (30 days before period start); period 01/03/2026-28/05/2026. "Repairs to lift (mis-use)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Argyle Locksmiths</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Charged 05/02/2026 (24 days before period start); period 01/03/2026-28/05/2026. "Lower car park door reset code"</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Charged 16/02/2026 (13 days before period start); period 01/03/2026-28/05/2026. "Repair to upper car park shutter"</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Charge date outside invoice period</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="n">
-        <v>-7.72</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Charged 29/05/2026 (1 days after period end); period 01/03/2026-28/05/2026. "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Credit / negative line</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1883739</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="n">
-        <v>-7.42</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>-7.42 — "E-billing Discount: 29/08/2025 - 28/11/2025"</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Credit / negative line</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>-1.03</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>-1.03 — "Attended site to program numbers as requested"</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Credit / negative line</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="n">
-        <v>-7.42</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>-7.42 — "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Credit / negative line</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="n">
-        <v>-7.72</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>-7.72 — "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Credit / negative line</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>ONESCO Ltd</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>-7.72</v>
+        <v>11.03</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>-7.72 — "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
+          <t>Service period 26/06/2025-17/07/2025 ends 43 days before the invoice quarter starts (29/08/2025). "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2"</t>
         </is>
       </c>
     </row>
@@ -10565,23 +10423,26 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>HDN- NIG - 2025-2026</t>
-        </is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" s="3" t="n">
+        <v>-228.33</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>'HDN- NIG - 2025-2026' billed in 2/3 prior quarters but is absent this quarter.</t>
+          <t>Electricity: 144.38 this quarter vs prior average 372.71 (0.4x, lower).</t>
         </is>
       </c>
     </row>
@@ -10593,23 +10454,26 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>VWS (UK) T/A Veolia Water Technologies</t>
-        </is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" s="3" t="n">
+        <v>-159.955</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>'VWS (UK) T/A Veolia Water Technologies' billed in 2/3 prior quarters but is absent this quarter.</t>
+          <t>Electricity: 98.59 this quarter vs prior average 258.54 (0.4x, lower).</t>
         </is>
       </c>
     </row>
@@ -10621,35 +10485,1121 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>Abnormal category total</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" s="3" t="n">
+        <v>-35.585</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Life System: 30.35 this quarter vs prior average 65.94 (0.5x, lower).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Abnormal category total</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" s="3" t="n">
+        <v>-77.255</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Repairs: 45.04 this quarter vs prior average 122.30 (0.4x, lower).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Abnormal category total</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" s="3" t="n">
+        <v>-120.6166666666667</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Electricity: 84.61 this quarter vs prior average 205.23 (0.4x, lower).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Abnormal vendor total</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ASD Electrical Contractors Ltd</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>-32.32</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>ASD Electrical Contractors Ltd: 2.26 this quarter vs prior average 34.58 (0.1x, lower).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Abnormal vendor total</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>42.92666666666666</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd: 81.91 this quarter vs prior average 38.98 (2.1x, higher).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Charged 30/04/2025 (29 days before period start); period 29/05/2025-28/08/2025. "Sim card charge for the GSM door access system: 01/04/2025 -"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Charged 23/05/2025 (6 days before period start); period 29/05/2025-28/08/2025. "Attended site and downloaded CCTV footage from mailbox camer"</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>80.28</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Charged 29/08/2025 (1 days after period end); period 29/05/2025-28/08/2025. "Management Fee: 29/08/2025 - 28/11/2025"</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>PTSG Electrical Services Ltd</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Charged 08/08/2025 (21 days before period start); period 29/08/2025-28/11/2025. "Test &amp; Inspection of the Lighting Protection System"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Charged 22/08/2025 (7 days before period start); period 29/08/2025-28/11/2025. "Door entry SIM card charge"</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>AB Decorators</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>22.29</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Charged 26/08/2025 (3 days before period start); period 29/08/2025-28/11/2025. "Repairs to floor 11, 4, 1 &amp; stairwell to ground"</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>-7.42</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025. "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>80.28</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025. "Management Fee: 29/11/2025 - 28/02/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Grounds</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Cleansite Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Charged 17/11/2025 (12 days before period start); period 29/11/2025-28/02/2026. "Bulk uplift"</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Ritchie Mackenzie &amp; Co Ltd</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Charged 31/10/2025 (29 days before period start); period 29/11/2025-28/02/2026. "Service checks on 1 x Two Pump Booster Set"</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Hart Lifts Ltd</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Charged 14/11/2025 (15 days before period start); period 29/11/2025-28/02/2026. "Repairs to lift controller unit"</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Hart Lifts Ltd</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Charged 21/11/2025 (8 days before period start); period 29/11/2025-28/02/2026. "Renewed damaged lift door spring"</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Integra Building Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Charged 25/11/2025 (4 days before period start); period 29/11/2025-28/02/2026. "Replace dry riser inlet lock"</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Charged 01/03/2026 (1 days after period end); period 29/11/2025-28/02/2026. "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Charged 31/01/2026 (29 days before period start); period 01/03/2026-28/05/2026. "Door entry SIM card charge"</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Charged 15/02/2026 (14 days before period start); period 01/03/2026-28/05/2026. "Reset fire alarm system"</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Hart Lifts Ltd</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Charged 30/01/2026 (30 days before period start); period 01/03/2026-28/05/2026. "Repairs to lift (mis-use)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Argyle Locksmiths</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Charged 05/02/2026 (24 days before period start); period 01/03/2026-28/05/2026. "Lower car park door reset code"</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Charged 16/02/2026 (13 days before period start); period 01/03/2026-28/05/2026. "Repair to upper car park shutter"</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Charge date outside invoice period</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Charged 29/05/2026 (1 days after period end); period 01/03/2026-28/05/2026. "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>-7.42</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>-7.42 — "E-billing Discount: 29/08/2025 - 28/11/2025"</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>-1.03 — "Attended site to program numbers as requested"</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>-7.42</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>-7.42 — "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>-7.72 — "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>-7.72 — "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Dropped vendor</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>HDN- NIG - 2025-2026</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>'HDN- NIG - 2025-2026' billed in 2/3 prior quarters but is absent this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Dropped vendor</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>VWS (UK) T/A Veolia Water Technologies</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>'VWS (UK) T/A Veolia Water Technologies' billed in 2/3 prior quarters but is absent this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>Stale service period</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>1883739</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>Life System</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F81" s="3" t="n">
         <v>0.29</v>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>Service period 01/04/2025-30/04/2025 ends 29 days before the invoice quarter starts (29/05/2025). "Sim card charge for the GSM door access system: 01"</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G49"/>
+  <autoFilter ref="A1:G81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update invoice skill to count anomolies
</commit_message>
<xml_diff>
--- a/.claude/skills/invoice-tracker/output/cost_tracker.xlsx
+++ b/.claude/skills/invoice-tracker/output/cost_tracker.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Line Items'!$A$1:$O$105</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anomalies'!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Anomalies'!$A$1:$G$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2487,73 +2487,77 @@
       <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>2025/26</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>1933254</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>14/11/2025</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>29/08/2025</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>28/11/2025</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Electricity</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>01/09/2025</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>Ecotricity DD</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>Common electricity supply 1: 01/04/2025 - 01/10/2025</t>
         </is>
       </c>
-      <c r="J26" s="3" t="n">
+      <c r="J26" s="9" t="n">
         <v>5053.31</v>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>1/35</t>
         </is>
       </c>
-      <c r="L26" s="3" t="n">
+      <c r="L26" s="9" t="n">
         <v>144.38</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M26" s="8" t="inlineStr">
         <is>
           <t>01/04/2025</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N26" s="8" t="inlineStr">
         <is>
           <t>01/10/2025</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" s="8" t="inlineStr">
+        <is>
+          <t>Cross-invoice duplicate charge</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2946,142 +2950,150 @@
       <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>2025/26</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>1933254</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>14/11/2025</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>29/08/2025</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>28/11/2025</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>Life System</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>30/09/2025</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="8" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Quarterly service and inspection of car park garage ventilation: 01/06/2025 - 30/09/2025</t>
         </is>
       </c>
-      <c r="J33" s="3" t="n">
+      <c r="J33" s="9" t="n">
         <v>94.2</v>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="8" t="inlineStr">
         <is>
           <t>1/18</t>
         </is>
       </c>
-      <c r="L33" s="3" t="n">
+      <c r="L33" s="9" t="n">
         <v>5.23</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33" s="8" t="inlineStr">
         <is>
           <t>01/06/2025</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N33" s="8" t="inlineStr">
         <is>
           <t>30/09/2025</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" s="8" t="inlineStr">
+        <is>
+          <t>Cross-invoice duplicate charge</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>2025/26</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>1933254</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>14/11/2025</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>29/08/2025</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>28/11/2025</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="8" t="inlineStr">
         <is>
           <t>Life System</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>30/09/2025</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="8" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="8" t="inlineStr">
         <is>
           <t>Quarterly smoke extract sys service: 01/06/2025 - 30/09/2025</t>
         </is>
       </c>
-      <c r="J34" s="3" t="n">
+      <c r="J34" s="9" t="n">
         <v>160.2</v>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="8" t="inlineStr">
         <is>
           <t>1/35</t>
         </is>
       </c>
-      <c r="L34" s="3" t="n">
+      <c r="L34" s="9" t="n">
         <v>4.57</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34" s="8" t="inlineStr">
         <is>
           <t>01/06/2025</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N34" s="8" t="inlineStr">
         <is>
           <t>30/09/2025</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" s="8" t="inlineStr">
+        <is>
+          <t>Cross-invoice duplicate charge</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4441,73 +4453,77 @@
       <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>2025/26</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>1968807</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="8" t="inlineStr">
         <is>
           <t>23/02/2026</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="8" t="inlineStr">
         <is>
           <t>29/11/2025</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="8" t="inlineStr">
         <is>
           <t>28/02/2026</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="8" t="inlineStr">
         <is>
           <t>Electricity</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="8" t="inlineStr">
         <is>
           <t>01/12/2025</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H56" s="8" t="inlineStr">
         <is>
           <t>Ecotricity DD</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I56" s="8" t="inlineStr">
         <is>
           <t>Common electricity supply 1: 01/06/2025 - 01/01/2026</t>
         </is>
       </c>
-      <c r="J56" s="3" t="n">
+      <c r="J56" s="9" t="n">
         <v>3450.99</v>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K56" s="8" t="inlineStr">
         <is>
           <t>1/35</t>
         </is>
       </c>
-      <c r="L56" s="3" t="n">
+      <c r="L56" s="9" t="n">
         <v>98.59</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="M56" s="8" t="inlineStr">
         <is>
           <t>01/06/2025</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
+      <c r="N56" s="8" t="inlineStr">
         <is>
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
+      <c r="O56" s="8" t="inlineStr">
+        <is>
+          <t>Cross-invoice duplicate charge</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6691,142 +6707,150 @@
       <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="8" t="inlineStr">
         <is>
           <t>2025/26</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t>2013624</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="8" t="inlineStr">
         <is>
           <t>15/05/2026</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" s="8" t="inlineStr">
         <is>
           <t>01/03/2026</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E90" s="8" t="inlineStr">
         <is>
           <t>28/05/2026</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F90" s="8" t="inlineStr">
         <is>
           <t>Life System</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr">
+      <c r="G90" s="8" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H90" s="8" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
+      <c r="I90" s="8" t="inlineStr">
         <is>
           <t>Quarterly car park shutter inspection: 24/12/2025 - 31/03/2026</t>
         </is>
       </c>
-      <c r="J90" s="3" t="n">
+      <c r="J90" s="9" t="n">
         <v>260.04</v>
       </c>
-      <c r="K90" t="inlineStr">
+      <c r="K90" s="8" t="inlineStr">
         <is>
           <t>1/18</t>
         </is>
       </c>
-      <c r="L90" s="3" t="n">
+      <c r="L90" s="9" t="n">
         <v>14.45</v>
       </c>
-      <c r="M90" t="inlineStr">
+      <c r="M90" s="8" t="inlineStr">
         <is>
           <t>24/12/2025</t>
         </is>
       </c>
-      <c r="N90" t="inlineStr">
+      <c r="N90" s="8" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr"/>
+      <c r="O90" s="8" t="inlineStr">
+        <is>
+          <t>Possible duplicate line (same invoice)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="8" t="inlineStr">
         <is>
           <t>2025/26</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="8" t="inlineStr">
         <is>
           <t>2013624</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="8" t="inlineStr">
         <is>
           <t>15/05/2026</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" s="8" t="inlineStr">
         <is>
           <t>01/03/2026</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E91" s="8" t="inlineStr">
         <is>
           <t>28/05/2026</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F91" s="8" t="inlineStr">
         <is>
           <t>Life System</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr">
+      <c r="G91" s="8" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="H91" s="8" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
+      <c r="I91" s="8" t="inlineStr">
         <is>
           <t>Quarterly car park shutter inspection x2: 24/12/2025 - 31/03/2026</t>
         </is>
       </c>
-      <c r="J91" s="3" t="n">
+      <c r="J91" s="9" t="n">
         <v>260.04</v>
       </c>
-      <c r="K91" t="inlineStr">
+      <c r="K91" s="8" t="inlineStr">
         <is>
           <t>1/18</t>
         </is>
       </c>
-      <c r="L91" s="3" t="n">
+      <c r="L91" s="9" t="n">
         <v>14.45</v>
       </c>
-      <c r="M91" t="inlineStr">
+      <c r="M91" s="8" t="inlineStr">
         <is>
           <t>24/12/2025</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr">
+      <c r="N91" s="8" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
+      <c r="O91" s="8" t="inlineStr">
+        <is>
+          <t>Possible duplicate line (same invoice)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8952,7 +8976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9032,7 +9056,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Charged 31/01/2024 (484 days before period start); period 29/05/2025-28/08/2025. "Common electricity supply : 12/10/2023 - 31/01/2024"</t>
+          <t>Charged 31/01/2024 (484 days before period start); period 29/05/2025-28/08/2025; £326.98. "Common electricity supply : 12/10/2023 - 31/01/2024"</t>
         </is>
       </c>
     </row>
@@ -9067,7 +9091,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Charged 31/08/2024 (271 days before period start); period 29/05/2025-28/08/2025. "vecon drive at pump"</t>
+          <t>Charged 31/08/2024 (271 days before period start); period 29/05/2025-28/08/2025; £56.27. "vecon drive at pump"</t>
         </is>
       </c>
     </row>
@@ -9102,7 +9126,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Charged 31/10/2024 (210 days before period start); period 29/05/2025-28/08/2025. "Service checks of 1 x booster set"</t>
+          <t>Charged 31/10/2024 (210 days before period start); period 29/05/2025-28/08/2025; £6.17. "Service checks of 1 x booster set"</t>
         </is>
       </c>
     </row>
@@ -9149,61 +9173,65 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Possible duplicate line (same invoice)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2x same vendor/period/cost with different descriptions: PTM Security Solutions Ltd 24/12/2025-31/03/2026 14.45 each — "Quarterly car park shutter inspection: 2" | "Quarterly car park shutter inspection x2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Stale service period</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>1883739</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Electricity</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>SSE Scottish Hydro - A/C 00000000</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F7" s="3" t="n">
         <v>326.98</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Service period 12/10/2023-31/01/2024 ends 484 days before the invoice quarter starts (29/05/2025). "Common electricity supply : 12/10/2023 - 31/01/202"</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Abnormal category total</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Maintenance</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" s="3" t="n">
-        <v>16.38</v>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Maintenance: 20.40 this quarter vs prior average 4.02 (5.1x, higher).</t>
+          <t>Service period 12/10/2023-31/01/2024 ends 484 days before the invoice quarter starts (29/05/2025); £326.98. "Common electricity supply : 12/10/2023 - 31/01/202"</t>
         </is>
       </c>
     </row>
@@ -9215,30 +9243,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>13.85</v>
+        <v>16.38</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Charged 23/04/2025 (36 days before period start); period 29/05/2025-28/08/2025. "Attended site to re-fit fan control cabinet to the wall: 26/"</t>
+          <t>Maintenance: 20.40 this quarter vs prior average 4.02 (5.1x, higher).</t>
         </is>
       </c>
     </row>
@@ -9255,7 +9279,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>1883739</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -9265,15 +9289,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-1.03</v>
+        <v>13.85</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Charged 01/07/2025 (59 days before period start); period 29/08/2025-28/11/2025. "Attended site to program numbers as requested"</t>
+          <t>Charged 23/04/2025 (36 days before period start); period 29/05/2025-28/08/2025; £13.85. "Attended site to re-fit fan control cabinet to the wall: 26/"</t>
         </is>
       </c>
     </row>
@@ -9300,15 +9324,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>3.4</v>
+        <v>-1.03</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Charged 15/07/2025 (45 days before period start); period 29/08/2025-28/11/2025. "Monitoring of CCTV"</t>
+          <t>Charged 01/07/2025 (59 days before period start); period 29/08/2025-28/11/2025; £-1.03. "Attended site to program numbers as requested"</t>
         </is>
       </c>
     </row>
@@ -9335,15 +9359,15 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ONESCO Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>11.03</v>
+        <v>3.4</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Charged 17/07/2025 (43 days before period start); period 29/08/2025-28/11/2025. "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2025"</t>
+          <t>Charged 15/07/2025 (45 days before period start); period 29/08/2025-28/11/2025; £3.40. "Monitoring of CCTV"</t>
         </is>
       </c>
     </row>
@@ -9360,25 +9384,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>ONESCO Ltd</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>86.5</v>
+        <v>11.03</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Charged 28/05/2026 (89 days after period end); period 29/11/2025-28/02/2026. "Management Fee: 01/03/2026 - 28/05/2026"</t>
+          <t>Charged 17/07/2025 (43 days before period start); period 29/08/2025-28/11/2025; £11.03. "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2025"</t>
         </is>
       </c>
     </row>
@@ -9395,25 +9419,25 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Life System</t>
+          <t>Management Fee</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.7</v>
+        <v>86.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Charged 17/12/2025 (74 days before period start); period 01/03/2026-28/05/2026. "Quarterly fire alarm service"</t>
+          <t>Charged 28/05/2026 (89 days after period end); period 29/11/2025-28/02/2026; £86.50. "Management Fee: 01/03/2026 - 28/05/2026"</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9459,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -9444,11 +9468,11 @@
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>1.03</v>
+        <v>2.7</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Charged 23/12/2025 (68 days before period start); period 01/03/2026-28/05/2026. "Door entry sim card change"</t>
+          <t>Charged 17/12/2025 (74 days before period start); period 01/03/2026-28/05/2026; £2.70. "Quarterly fire alarm service"</t>
         </is>
       </c>
     </row>
@@ -9475,15 +9499,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ritchie Mackenzie &amp; Co Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>58.58</v>
+        <v>1.03</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Charged 28/01/2026 (32 days before period start); period 01/03/2026-28/05/2026. "Attended site to install new pump to replace missing pump"</t>
+          <t>Charged 23/12/2025 (68 days before period start); period 01/03/2026-28/05/2026; £1.03. "Door entry sim card change"</t>
         </is>
       </c>
     </row>
@@ -9505,20 +9529,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>Ritchie Mackenzie &amp; Co Ltd</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>86.5</v>
+        <v>58.58</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Charged 28/08/2026 (92 days after period end); period 01/03/2026-28/05/2026. "Management Fee: 29/05/2026 - 28/08/2026"</t>
+          <t>Charged 28/01/2026 (32 days before period start); period 01/03/2026-28/05/2026; £58.58. "Attended site to install new pump to replace missing pump"</t>
         </is>
       </c>
     </row>
@@ -9530,23 +9554,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HDN- NIG - 2025-2026</t>
-        </is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>86.5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>'HDN- NIG - 2025-2026' billed in 2/2 prior quarters but is absent this quarter.</t>
+          <t>Charged 28/08/2026 (92 days after period end); period 01/03/2026-28/05/2026; £86.50. "Management Fee: 29/05/2026 - 28/08/2026"</t>
         </is>
       </c>
     </row>
@@ -9558,23 +9589,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Cross-invoice duplicate charge</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ASD Electrical Contractors Ltd</t>
-        </is>
+          <t>Ecotricity DD</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>144.38</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>'ASD Electrical Contractors Ltd' billed in 3/3 prior quarters but is absent this quarter.</t>
+          <t>Ecotricity DD: service 01/04/2025-01/10/2025 overlaps 92d with inv 1883739 15/03/2025-01/07/2025; £144.38. "Common electricity supply 1: 01/04/2025 " vs "Common electricity supply 1: 15/03/2025 "</t>
         </is>
       </c>
     </row>
@@ -9586,7 +9624,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New vendor</t>
+          <t>Cross-invoice duplicate charge</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9594,18 +9632,22 @@
           <t>1933254</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AB Decorators</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>22.29</v>
+        <v>5.23</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>'AB Decorators' appears this quarter but not in any prior quarter (cost 22.29).</t>
+          <t>PTM Security Solutions Ltd: service 01/06/2025-30/09/2025 overlaps 36d with inv 1883739 26/06/2025-31/07/2025; £5.23. "Quarterly service and inspection of car " vs "Door entry SIM card charge: 26/06/2025 -"</t>
         </is>
       </c>
     </row>
@@ -9617,7 +9659,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>New vendor</t>
+          <t>Cross-invoice duplicate charge</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -9625,18 +9667,22 @@
           <t>1933254</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Columbus Facilities Maintenance Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>18.85</v>
+        <v>5.23</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>'Columbus Facilities Maintenance Ltd' appears this quarter but not in any prior quarter (cost 18.85).</t>
+          <t>PTM Security Solutions Ltd: service 01/06/2025-30/09/2025 overlaps 122d with inv 1883739 01/06/2025-30/09/2025; £5.23. "Quarterly service and inspection of car " vs "Quarterly service and inspection car par"</t>
         </is>
       </c>
     </row>
@@ -9648,26 +9694,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New vendor</t>
+          <t>Cross-invoice duplicate charge</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Hart Lifts Ltd</t>
+          <t>Ecotricity DD</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>7.52</v>
+        <v>98.59</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>'Hart Lifts Ltd' appears this quarter but not in any prior quarter (cost 7.52).</t>
+          <t>Ecotricity DD: service 01/06/2025-01/01/2026 overlaps 123d with inv 1933254 01/04/2025-01/10/2025; £98.59. "Common electricity supply 1: 01/06/2025 " vs "Common electricity supply 1: 01/04/2025 "</t>
         </is>
       </c>
     </row>
@@ -9679,26 +9729,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New vendor</t>
+          <t>Dropped vendor</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Integra Building Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>2.23</v>
+          <t>HDN- NIG - 2025-2026</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>'Integra Building Solutions Ltd' appears this quarter but not in any prior quarter (cost 2.23).</t>
+          <t>'HDN- NIG - 2025-2026' billed in 2/2 prior quarters but is absent this quarter.</t>
         </is>
       </c>
     </row>
@@ -9710,26 +9757,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New vendor</t>
+          <t>Dropped vendor</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>2013624</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ONESCO Ltd</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>44.27</v>
+          <t>ASD Electrical Contractors Ltd</t>
+        </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>'ONESCO Ltd' appears this quarter but not in any prior quarter (cost 44.27).</t>
+          <t>'ASD Electrical Contractors Ltd' billed in 3/3 prior quarters but is absent this quarter.</t>
         </is>
       </c>
     </row>
@@ -9752,15 +9796,15 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PTSG Electrical Services Ltd</t>
+          <t>AB Decorators</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>22.94</v>
+        <v>22.29</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>'PTSG Electrical Services Ltd' appears this quarter but not in any prior quarter (cost 22.94).</t>
+          <t>'AB Decorators' appears this quarter but not in any prior quarter (cost 22.29).</t>
         </is>
       </c>
     </row>
@@ -9777,21 +9821,21 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>APS Safety Systems Limited</t>
+          <t>Columbus Facilities Maintenance Ltd</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>10.51</v>
+        <v>18.85</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>'APS Safety Systems Limited' appears this quarter but not in any prior quarter (cost 10.51).</t>
+          <t>'Columbus Facilities Maintenance Ltd' appears this quarter but not in any prior quarter (cost 18.85).</t>
         </is>
       </c>
     </row>
@@ -9808,21 +9852,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>City Drain Clear</t>
+          <t>Hart Lifts Ltd</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>3.34</v>
+        <v>7.52</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>'City Drain Clear' appears this quarter but not in any prior quarter (cost 3.34).</t>
+          <t>'Hart Lifts Ltd' appears this quarter but not in any prior quarter (cost 7.52).</t>
         </is>
       </c>
     </row>
@@ -9839,21 +9883,21 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Cleansite Solutions Ltd</t>
+          <t>Integra Building Solutions Ltd</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5.15</v>
+        <v>2.23</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>'Cleansite Solutions Ltd' appears this quarter but not in any prior quarter (cost 5.15).</t>
+          <t>'Integra Building Solutions Ltd' appears this quarter but not in any prior quarter (cost 2.23).</t>
         </is>
       </c>
     </row>
@@ -9870,21 +9914,21 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DAWN ZURICH 26/27</t>
+          <t>ONESCO Ltd</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>11.43</v>
+        <v>44.27</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>'DAWN ZURICH 26/27' appears this quarter but not in any prior quarter (cost 11.43).</t>
+          <t>'ONESCO Ltd' appears this quarter but not in any prior quarter (cost 44.27).</t>
         </is>
       </c>
     </row>
@@ -9901,21 +9945,21 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DAWN- INTACT-26-27</t>
+          <t>PTSG Electrical Services Ltd</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>181.01</v>
+        <v>22.94</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>'DAWN- INTACT-26-27' appears this quarter but not in any prior quarter (cost 181.01).</t>
+          <t>'PTSG Electrical Services Ltd' appears this quarter but not in any prior quarter (cost 22.94).</t>
         </is>
       </c>
     </row>
@@ -9938,15 +9982,15 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>J.T. Mullen Building Services</t>
+          <t>APS Safety Systems Limited</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>3.77</v>
+        <v>10.51</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>'J.T. Mullen Building Services' appears this quarter but not in any prior quarter (cost 3.77).</t>
+          <t>'APS Safety Systems Limited' appears this quarter but not in any prior quarter (cost 10.51).</t>
         </is>
       </c>
     </row>
@@ -9963,21 +10007,21 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Argyle Locksmiths</t>
+          <t>City Drain Clear</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>2.71</v>
+        <v>3.34</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>'Argyle Locksmiths' appears this quarter but not in any prior quarter (cost 2.71).</t>
+          <t>'City Drain Clear' appears this quarter but not in any prior quarter (cost 3.34).</t>
         </is>
       </c>
     </row>
@@ -9989,23 +10033,26 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Recurring item missing</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Cleansite Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>5.15</v>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>'attended site and downloaded cctv footage from mailbox camera' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'Cleansite Solutions Ltd' appears this quarter but not in any prior quarter (cost 5.15).</t>
         </is>
       </c>
     </row>
@@ -10017,23 +10064,26 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Recurring item missing</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>DAWN ZURICH 26/27</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>11.43</v>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>'attended site and removed snib from fire door dry riser door was detached from wall so attached timber batons to secure door' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'DAWN ZURICH 26/27' appears this quarter but not in any prior quarter (cost 11.43).</t>
         </is>
       </c>
     </row>
@@ -10045,23 +10095,26 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Recurring item missing</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>DAWN- INTACT-26-27</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>181.01</v>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>'attended site to re fit fan control cabinet to the wall' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'DAWN- INTACT-26-27' appears this quarter but not in any prior quarter (cost 181.01).</t>
         </is>
       </c>
     </row>
@@ -10073,23 +10126,26 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Recurring item missing</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>J.T. Mullen Building Services</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>3.77</v>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>'emergency lighting repair' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'J.T. Mullen Building Services' appears this quarter but not in any prior quarter (cost 3.77).</t>
         </is>
       </c>
     </row>
@@ -10101,23 +10157,26 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Recurring item missing</t>
+          <t>New vendor</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Argyle Locksmiths</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>2.71</v>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>'quarterly service and inspection car park garage shutter' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'Argyle Locksmiths' appears this quarter but not in any prior quarter (cost 2.71).</t>
         </is>
       </c>
     </row>
@@ -10139,13 +10198,13 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>'replace faulty ball valves' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'attended site and downloaded cctv footage from mailbox camera' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10173,7 +10232,7 @@
       <c r="E38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>'service checks of x booster set' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'attended site and removed snib from fire door dry riser door was detached from wall so attached timber batons to secure door' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10195,13 +10254,13 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Life System</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>'sim card charge for the gsm door access system' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'attended site to re fit fan control cabinet to the wall' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10229,7 +10288,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>'sim card charges for gsm door access system' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'emergency lighting repair' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10257,7 +10316,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>'vecon drive at pump' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'quarterly service and inspection car park garage shutter' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10279,13 +10338,13 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Life System</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>'water testing certification' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+          <t>'replace faulty ball valves' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10361,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -10313,7 +10372,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>'attended site to program numbers as requested' (e.g. Repairs) appeared in all 2 prior quarters but not this quarter.</t>
+          <t>'service checks of x booster set' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10330,7 +10389,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -10341,7 +10400,7 @@
       <c r="E44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>'quarterly fire alarm service' (e.g. Life System) appeared in all 2 prior quarters but not this quarter.</t>
+          <t>'sim card charge for the gsm door access system' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10353,30 +10412,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Stale service period</t>
+          <t>Recurring item missing</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="n">
-        <v>13.85</v>
-      </c>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Service period 26/03/2025-23/04/2025 ends 36 days before the invoice quarter starts (29/05/2025). "Attended site to re-fit fan control cabinet to the"</t>
+          <t>'sim card charges for gsm door access system' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
         </is>
       </c>
     </row>
@@ -10388,185 +10440,177 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>'vecon drive at pump' (e.g. Repairs) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>'water testing certification' (e.g. Life System) appeared in all 1 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>'attended site to program numbers as requested' (e.g. Repairs) appeared in all 2 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Recurring item missing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Life System</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>'quarterly fire alarm service' (e.g. Life System) appeared in all 2 prior quarters but not this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>Stale service period</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>PTM Security Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Service period 26/03/2025-23/04/2025 ends 36 days before the invoice quarter starts (29/05/2025); £13.85. "Attended site to re-fit fan control cabinet to the"</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Stale service period</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
         <is>
           <t>1933254</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Repairs</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>ONESCO Ltd</t>
         </is>
       </c>
-      <c r="F46" s="3" t="n">
+      <c r="F51" s="3" t="n">
         <v>11.03</v>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Service period 26/06/2025-17/07/2025 ends 43 days before the invoice quarter starts (29/08/2025). "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2"</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Abnormal category total</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Electricity</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" s="3" t="n">
-        <v>-228.33</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Electricity: 144.38 this quarter vs prior average 372.71 (0.4x, lower).</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Abnormal category total</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Electricity</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" s="3" t="n">
-        <v>-159.955</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Electricity: 98.59 this quarter vs prior average 258.54 (0.4x, lower).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Abnormal category total</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" s="3" t="n">
-        <v>-35.585</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Life System: 30.35 this quarter vs prior average 65.94 (0.5x, lower).</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Abnormal category total</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Repairs</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" s="3" t="n">
-        <v>-77.255</v>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Repairs: 45.04 this quarter vs prior average 122.30 (0.4x, lower).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Abnormal category total</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Electricity</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" s="3" t="n">
-        <v>-120.6166666666667</v>
-      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Electricity: 84.61 this quarter vs prior average 205.23 (0.4x, lower).</t>
+          <t>Service period 26/06/2025-17/07/2025 ends 43 days before the invoice quarter starts (29/08/2025); £11.03. "Trace &amp; locate water ingress: 26/06/2025 - 17/07/2"</t>
         </is>
       </c>
     </row>
@@ -10578,26 +10622,26 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Abnormal vendor total</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1968807</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>ASD Electrical Contractors Ltd</t>
-        </is>
-      </c>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" s="3" t="n">
-        <v>-32.32</v>
+        <v>-228.33</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>ASD Electrical Contractors Ltd: 2.26 this quarter vs prior average 34.58 (0.1x, lower).</t>
+          <t>Electricity: 144.38 this quarter vs prior average 372.71 (0.4x, lower).</t>
         </is>
       </c>
     </row>
@@ -10609,26 +10653,26 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Abnormal vendor total</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" s="3" t="n">
-        <v>42.92666666666666</v>
+        <v>-159.955</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd: 81.91 this quarter vs prior average 38.98 (2.1x, higher).</t>
+          <t>Electricity: 98.59 this quarter vs prior average 258.54 (0.4x, lower).</t>
         </is>
       </c>
     </row>
@@ -10640,12 +10684,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -10653,17 +10697,13 @@
           <t>Life System</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
       <c r="F54" s="3" t="n">
-        <v>0.29</v>
+        <v>-35.585</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Charged 30/04/2025 (29 days before period start); period 29/05/2025-28/08/2025. "Sim card charge for the GSM door access system: 01/04/2025 -"</t>
+          <t>Life System: 30.35 this quarter vs prior average 65.94 (0.5x, lower).</t>
         </is>
       </c>
     </row>
@@ -10675,30 +10715,26 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Life System</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>PTM Security Solutions Ltd</t>
-        </is>
-      </c>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" s="3" t="n">
-        <v>4.25</v>
+        <v>-77.255</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Charged 23/05/2025 (6 days before period start); period 29/05/2025-28/08/2025. "Attended site and downloaded CCTV footage from mailbox camer"</t>
+          <t>Repairs: 45.04 this quarter vs prior average 122.30 (0.4x, lower).</t>
         </is>
       </c>
     </row>
@@ -10710,30 +10746,26 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal category total</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>2013624</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Management Fee</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Newton Property Management Ltd</t>
-        </is>
-      </c>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" s="3" t="n">
-        <v>80.28</v>
+        <v>-120.6166666666667</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Charged 29/08/2025 (1 days after period end); period 29/05/2025-28/08/2025. "Management Fee: 29/08/2025 - 28/11/2025"</t>
+          <t>Electricity: 84.61 this quarter vs prior average 205.23 (0.4x, lower).</t>
         </is>
       </c>
     </row>
@@ -10745,30 +10777,26 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal vendor total</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>PTSG Electrical Services Ltd</t>
+          <t>ASD Electrical Contractors Ltd</t>
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>7.2</v>
+        <v>-32.32</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Charged 08/08/2025 (21 days before period start); period 29/08/2025-28/11/2025. "Test &amp; Inspection of the Lighting Protection System"</t>
+          <t>ASD Electrical Contractors Ltd: 2.26 this quarter vs prior average 34.58 (0.1x, lower).</t>
         </is>
       </c>
     </row>
@@ -10780,30 +10808,26 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Charge date outside invoice period</t>
+          <t>Abnormal vendor total</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1933254</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Life System</t>
-        </is>
-      </c>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F58" s="3" t="n">
-        <v>0.3</v>
+        <v>42.92666666666666</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Charged 22/08/2025 (7 days before period start); period 29/08/2025-28/11/2025. "Door entry SIM card charge"</t>
+          <t>PTM Security Solutions Ltd: 81.91 this quarter vs prior average 38.98 (2.1x, higher).</t>
         </is>
       </c>
     </row>
@@ -10820,25 +10844,25 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>1883739</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>AB Decorators</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>22.29</v>
+        <v>0.29</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Charged 26/08/2025 (3 days before period start); period 29/08/2025-28/11/2025. "Repairs to floor 11, 4, 1 &amp; stairwell to ground"</t>
+          <t>Charged 30/04/2025 (29 days before period start); period 29/05/2025-28/08/2025; £0.29. "Sim card charge for the GSM door access system: 01/04/2025 -"</t>
         </is>
       </c>
     </row>
@@ -10855,25 +10879,25 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>1883739</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F60" s="3" t="n">
-        <v>-7.42</v>
+        <v>4.25</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025. "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
+          <t>Charged 23/05/2025 (6 days before period start); period 29/05/2025-28/08/2025; £4.25. "Attended site and downloaded CCTV footage from mailbox camer"</t>
         </is>
       </c>
     </row>
@@ -10890,7 +10914,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>1883739</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -10908,7 +10932,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025. "Management Fee: 29/11/2025 - 28/02/2026"</t>
+          <t>Charged 29/08/2025 (1 days after period end); period 29/05/2025-28/08/2025; £80.28. "Management Fee: 29/08/2025 - 28/11/2025"</t>
         </is>
       </c>
     </row>
@@ -10925,25 +10949,25 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Grounds</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Cleansite Solutions Ltd</t>
+          <t>PTSG Electrical Services Ltd</t>
         </is>
       </c>
       <c r="F62" s="3" t="n">
-        <v>5.15</v>
+        <v>7.2</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Charged 17/11/2025 (12 days before period start); period 29/11/2025-28/02/2026. "Bulk uplift"</t>
+          <t>Charged 08/08/2025 (21 days before period start); period 29/08/2025-28/11/2025; £7.20. "Test &amp; Inspection of the Lighting Protection System"</t>
         </is>
       </c>
     </row>
@@ -10960,25 +10984,25 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Ritchie Mackenzie &amp; Co Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>5.83</v>
+        <v>0.3</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Charged 31/10/2025 (29 days before period start); period 29/11/2025-28/02/2026. "Service checks on 1 x Two Pump Booster Set"</t>
+          <t>Charged 22/08/2025 (7 days before period start); period 29/08/2025-28/11/2025; £0.30. "Door entry SIM card charge"</t>
         </is>
       </c>
     </row>
@@ -10995,7 +11019,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -11005,15 +11029,15 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Hart Lifts Ltd</t>
+          <t>AB Decorators</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
-        <v>8.33</v>
+        <v>22.29</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Charged 14/11/2025 (15 days before period start); period 29/11/2025-28/02/2026. "Repairs to lift controller unit"</t>
+          <t>Charged 26/08/2025 (3 days before period start); period 29/08/2025-28/11/2025; £22.29. "Repairs to floor 11, 4, 1 &amp; stairwell to ground"</t>
         </is>
       </c>
     </row>
@@ -11030,25 +11054,25 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Management Fee</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Hart Lifts Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>5.48</v>
+        <v>-7.42</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Charged 21/11/2025 (8 days before period start); period 29/11/2025-28/02/2026. "Renewed damaged lift door spring"</t>
+          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025; £-7.42. "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
         </is>
       </c>
     </row>
@@ -11065,25 +11089,25 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>1933254</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Management Fee</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Integra Building Solutions Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F66" s="3" t="n">
-        <v>2.57</v>
+        <v>80.28</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Charged 25/11/2025 (4 days before period start); period 29/11/2025-28/02/2026. "Replace dry riser inlet lock"</t>
+          <t>Charged 29/11/2025 (1 days after period end); period 29/08/2025-28/11/2025; £80.28. "Management Fee: 29/11/2025 - 28/02/2026"</t>
         </is>
       </c>
     </row>
@@ -11105,20 +11129,20 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Grounds</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>Cleansite Solutions Ltd</t>
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>-7.72</v>
+        <v>5.15</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Charged 01/03/2026 (1 days after period end); period 29/11/2025-28/02/2026. "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
+          <t>Charged 17/11/2025 (12 days before period start); period 29/11/2025-28/02/2026; £5.15. "Bulk uplift"</t>
         </is>
       </c>
     </row>
@@ -11135,25 +11159,25 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Life System</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Ritchie Mackenzie &amp; Co Ltd</t>
         </is>
       </c>
       <c r="F68" s="3" t="n">
-        <v>0.31</v>
+        <v>5.83</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Charged 31/01/2026 (29 days before period start); period 01/03/2026-28/05/2026. "Door entry SIM card charge"</t>
+          <t>Charged 31/10/2025 (29 days before period start); period 29/11/2025-28/02/2026; £5.83. "Service checks on 1 x Two Pump Booster Set"</t>
         </is>
       </c>
     </row>
@@ -11170,25 +11194,25 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Life System</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Hart Lifts Ltd</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>5.53</v>
+        <v>8.33</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Charged 15/02/2026 (14 days before period start); period 01/03/2026-28/05/2026. "Reset fire alarm system"</t>
+          <t>Charged 14/11/2025 (15 days before period start); period 29/11/2025-28/02/2026; £8.33. "Repairs to lift controller unit"</t>
         </is>
       </c>
     </row>
@@ -11205,7 +11229,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -11219,11 +11243,11 @@
         </is>
       </c>
       <c r="F70" s="3" t="n">
-        <v>4.6</v>
+        <v>5.48</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Charged 30/01/2026 (30 days before period start); period 01/03/2026-28/05/2026. "Repairs to lift (mis-use)"</t>
+          <t>Charged 21/11/2025 (8 days before period start); period 29/11/2025-28/02/2026; £5.48. "Renewed damaged lift door spring"</t>
         </is>
       </c>
     </row>
@@ -11240,7 +11264,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -11250,15 +11274,15 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Argyle Locksmiths</t>
+          <t>Integra Building Solutions Ltd</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
-        <v>2.71</v>
+        <v>2.57</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Charged 05/02/2026 (24 days before period start); period 01/03/2026-28/05/2026. "Lower car park door reset code"</t>
+          <t>Charged 25/11/2025 (4 days before period start); period 29/11/2025-28/02/2026; £2.57. "Replace dry riser inlet lock"</t>
         </is>
       </c>
     </row>
@@ -11275,25 +11299,25 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2013624</t>
+          <t>1968807</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Repairs</t>
+          <t>Management Fee</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>PTM Security Solutions Ltd</t>
+          <t>Newton Property Management Ltd</t>
         </is>
       </c>
       <c r="F72" s="3" t="n">
-        <v>13.2</v>
+        <v>-7.72</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Charged 16/02/2026 (13 days before period start); period 01/03/2026-28/05/2026. "Repair to upper car park shutter"</t>
+          <t>Charged 01/03/2026 (1 days after period end); period 29/11/2025-28/02/2026; £-7.72. "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
         </is>
       </c>
     </row>
@@ -11315,20 +11339,20 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>-7.72</v>
+        <v>0.31</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Charged 29/05/2026 (1 days after period end); period 01/03/2026-28/05/2026. "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
+          <t>Charged 31/01/2026 (29 days before period start); period 01/03/2026-28/05/2026; £0.31. "Door entry SIM card charge"</t>
         </is>
       </c>
     </row>
@@ -11340,30 +11364,30 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Credit / negative line</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>1883739</t>
+          <t>2013624</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Life System</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F74" s="3" t="n">
-        <v>-7.42</v>
+        <v>5.53</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>-7.42 — "E-billing Discount: 29/08/2025 - 28/11/2025"</t>
+          <t>Charged 15/02/2026 (14 days before period start); period 01/03/2026-28/05/2026; £5.53. "Reset fire alarm system"</t>
         </is>
       </c>
     </row>
@@ -11375,12 +11399,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Credit / negative line</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>2013624</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -11390,15 +11414,15 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>Hart Lifts Ltd</t>
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>-1.03</v>
+        <v>4.6</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>-1.03 — "Attended site to program numbers as requested"</t>
+          <t>Charged 30/01/2026 (30 days before period start); period 01/03/2026-28/05/2026; £4.60. "Repairs to lift (mis-use)"</t>
         </is>
       </c>
     </row>
@@ -11410,30 +11434,30 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Credit / negative line</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>1933254</t>
+          <t>2013624</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>Argyle Locksmiths</t>
         </is>
       </c>
       <c r="F76" s="3" t="n">
-        <v>-7.42</v>
+        <v>2.71</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>-7.42 — "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
+          <t>Charged 05/02/2026 (24 days before period start); period 01/03/2026-28/05/2026; £2.71. "Lower car park door reset code"</t>
         </is>
       </c>
     </row>
@@ -11445,30 +11469,30 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Credit / negative line</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>1968807</t>
+          <t>2013624</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Management Fee</t>
+          <t>Repairs</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Newton Property Management Ltd</t>
+          <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>-7.72</v>
+        <v>13.2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>-7.72 — "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
+          <t>Charged 16/02/2026 (13 days before period start); period 01/03/2026-28/05/2026; £13.20. "Repair to upper car park shutter"</t>
         </is>
       </c>
     </row>
@@ -11480,7 +11504,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Credit / negative line</t>
+          <t>Charge date outside invoice period</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -11503,7 +11527,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>-7.72 — "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
+          <t>Charged 29/05/2026 (1 days after period end); period 01/03/2026-28/05/2026; £-7.72. "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
         </is>
       </c>
     </row>
@@ -11515,23 +11539,30 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Credit / negative line</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
+          <t>1883739</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>HDN- NIG - 2025-2026</t>
-        </is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>-7.42</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>'HDN- NIG - 2025-2026' billed in 2/3 prior quarters but is absent this quarter.</t>
+          <t>-7.42 — "E-billing Discount: 29/08/2025 - 28/11/2025"</t>
         </is>
       </c>
     </row>
@@ -11543,23 +11574,30 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Dropped vendor</t>
+          <t>Credit / negative line</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2013624</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>VWS (UK) T/A Veolia Water Technologies</t>
-        </is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>-1.03</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>'VWS (UK) T/A Veolia Water Technologies' billed in 2/3 prior quarters but is absent this quarter.</t>
+          <t>-1.03 — "Attended site to program numbers as requested"</t>
         </is>
       </c>
     </row>
@@ -11571,35 +11609,196 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>1933254</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>-7.42</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>-7.42 — "E-billing Discount: 29/11/2025 - 28/02/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>1968807</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>-7.72 — "E-billing Discount: 01/03/2026 - 28/05/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Credit / negative line</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Newton Property Management Ltd</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>-7.72</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>-7.72 — "E-billing Discount: 29/05/2026 - 28/08/2026"</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Dropped vendor</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>HDN- NIG - 2025-2026</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>'HDN- NIG - 2025-2026' billed in 2/3 prior quarters but is absent this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Dropped vendor</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2013624</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>VWS (UK) T/A Veolia Water Technologies</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>'VWS (UK) T/A Veolia Water Technologies' billed in 2/3 prior quarters but is absent this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
           <t>Stale service period</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>1883739</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>Life System</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>PTM Security Solutions Ltd</t>
         </is>
       </c>
-      <c r="F81" s="3" t="n">
+      <c r="F86" s="3" t="n">
         <v>0.29</v>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Service period 01/04/2025-30/04/2025 ends 29 days before the invoice quarter starts (29/05/2025). "Sim card charge for the GSM door access system: 01"</t>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Service period 01/04/2025-30/04/2025 ends 29 days before the invoice quarter starts (29/05/2025); £0.29. "Sim card charge for the GSM door access system: 01"</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:G86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>